<commit_message>
Cambie conectividad a pcmpi
</commit_message>
<xml_diff>
--- a/Bitacora.xlsx
+++ b/Bitacora.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\OneDrive\Escritorio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\OneDrive\Escritorio\TESIS 1ERA ENTREGA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3256CB1-62CE-4135-92C6-32DF55E878C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1180DF85-2BDC-4188-B509-CA2E30D16731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30300" yWindow="1155" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t>Semana N°1 Lunes 09/mar viernes 13/mar</t>
   </si>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>Sí</t>
+  </si>
+  <si>
+    <t>ok</t>
   </si>
 </sst>
 </file>
@@ -444,7 +447,7 @@
   <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -508,7 +511,9 @@
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="1"/>
+      <c r="B8" s="1" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">

</xml_diff>